<commit_message>
Add 24 Veins-of-the-Earth setting assets
New Assets-sheet section with 6 Force, 6 Cunning, 6 Wealth and 6 Magic
assets keyed to specific factions: Knotsmen pact-vaults and demonic
notaries, Aelf-Adal dream-walkers and Black Glass dream-knights,
Funginid spore-wreaths and cathedral choirs, dErO crystal mines and
lancers, Gnonmen lantern wardens and hearth-shrines, Substratal
stone-eaters and tribute stones, Deep Janeen maze-tolls and
aesthete-spies, and Olm listeners, larders and anatomists. Each entry
follows the standard WWN stat block (Cost / HP / attack line / counter /
min-attribute / traits / special). Faction rosters updated to feature
the relevant flavour assets so they appear in play immediately.
</commit_message>
<xml_diff>
--- a/WWN_Veins_of_the_Earth_Factions.xlsx
+++ b/WWN_Veins_of_the_Earth_Factions.xlsx
@@ -1146,7 +1146,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Spies</t>
+          <t>Dream-Walkers</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1155,19 +1155,19 @@
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>C vs C</t>
+          <t>C vs M</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>1d6</t>
+          <t>1d8</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Cunning 2</t>
+          <t>Cunning 3, Magic 2</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -1386,7 +1386,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Knights / Champions</t>
+          <t>Dream-Knights of the Black Glass Court</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -1395,14 +1395,14 @@
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>F vs F</t>
+          <t>F vs C</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Force 5</t>
+          <t>Force 5, Magic 2</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -1434,7 +1434,7 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Living Idol</t>
+          <t>Dream Anchor</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1455,17 +1455,17 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
           <t>1d8</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>1d6</t>
-        </is>
-      </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>Magic 3</t>
+          <t>Magic 4</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -1993,23 +1993,23 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Spirit Walkers</t>
+          <t>Spore-Wreaths</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Magic</t>
+          <t>Cunning</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D28" s="6" t="n">
         <v>6</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>M vs C</t>
+          <t>C vs C</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Magic 2</t>
+          <t>Cunning 2</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -2034,35 +2034,35 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Spore-Cathedral</t>
+          <t>Every slave market</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Saboteurs</t>
+          <t>Spore-Maddened Slaves</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Cunning</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>C vs W</t>
+          <t>F vs F</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>2d4</t>
+          <t>1d6</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -2072,12 +2072,12 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Cunning 2</t>
+          <t>Force 2</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Subtle</t>
+          <t>Fanatic</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
@@ -2089,7 +2089,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Death Cult</t>
+          <t>Spore-Cathedral Choir</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -2098,87 +2098,87 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>M vs C</t>
+          <t>M vs M</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
+          <t>1d8</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
           <t>1d6</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>1d4</t>
-        </is>
-      </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Magic 2</t>
+          <t>Magic 3</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>Subtle</t>
+          <t>Special</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Carrion grounds</t>
+          <t>Spore-Cathedral</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Informers</t>
+          <t>Death Cult</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Cunning</t>
+          <t>Magic</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>C vs C</t>
+          <t>M vs C</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
           <t>1d4</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Cunning 1</t>
+          <t>Magic 2</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Stealthed, Special</t>
+          <t>Subtle</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Every slave market</t>
+          <t>Carrion grounds</t>
         </is>
       </c>
     </row>
@@ -2744,38 +2744,38 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Magic Workshop</t>
+          <t>Crystal Mines</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Magic</t>
+          <t>Wealth</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D28" s="6" t="n">
         <v>10</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>W vs F</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1d6</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1d6</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Magic 2</t>
+          <t>Wealth 3, Magic 1</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -2785,14 +2785,14 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Buzzing Halls</t>
+          <t>Crystal Pylons</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Battle Mages</t>
+          <t>Crystal Lancers</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -2801,14 +2801,14 @@
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>8</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>F vs F</t>
+          <t>F vs M</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -2936,48 +2936,48 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Light Cavalry</t>
+          <t>Magic Workshop</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Magic</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>F vs F</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>1d8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>1d6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Force 3</t>
+          <t>Magic 2</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Special</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Mech-trolley tunnels</t>
+          <t>Buzzing Halls</t>
         </is>
       </c>
     </row>
@@ -4294,7 +4294,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Militia</t>
+          <t>Lantern Wardens</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -4303,34 +4303,34 @@
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>F vs F</t>
+          <t>F vs M</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
+          <t>1d8</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
           <t>1d4</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>1d4</t>
-        </is>
-      </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Force 1</t>
+          <t>Force 3</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Special</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
@@ -4342,7 +4342,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Light Cavalry</t>
+          <t>Tunnel Crawlers</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -4351,10 +4351,10 @@
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
@@ -4363,17 +4363,17 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>1d8</t>
+          <t>1d6</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>1d6</t>
+          <t>1d4</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Force 3</t>
+          <t>Force 2</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -4438,7 +4438,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Farmers</t>
+          <t>Mushroom Fields</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -4447,10 +4447,10 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
@@ -4469,7 +4469,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Wealth 1</t>
+          <t>Wealth 2</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -4479,14 +4479,14 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Mushroom fields</t>
+          <t>Surface of the Lantern Holds</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Hedge Mages</t>
+          <t>Hearth-Lantern Shrine</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -4495,10 +4495,10 @@
         </is>
       </c>
       <c r="C31" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
@@ -4517,12 +4517,12 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Magic 1</t>
+          <t>Magic 2</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Special</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
@@ -4534,7 +4534,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Informers</t>
+          <t>Lightless Cartographers</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -4543,10 +4543,10 @@
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
@@ -4570,7 +4570,7 @@
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Stealthed, Special</t>
+          <t>Stealthed, Mobile</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
@@ -5093,7 +5093,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Bound Spirit</t>
+          <t>Stone-Voice Oracle</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -5102,14 +5102,14 @@
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>M vs F</t>
+          <t>M vs M</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -5119,17 +5119,17 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>1d6</t>
+          <t>1d8</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Magic 3</t>
+          <t>Magic 4</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Special</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
@@ -5141,38 +5141,38 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Living Idol</t>
+          <t>Stone-Eaters</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Magic</t>
+          <t>Force</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D28" s="6" t="n">
         <v>14</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>M vs M</t>
+          <t>F vs F</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
+          <t>1d10</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
           <t>1d8</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>1d6</t>
-        </is>
-      </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Magic 3</t>
+          <t>Force 4, Magic 2</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -5189,48 +5189,48 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Pretorian Guard</t>
+          <t>Substratal Tribute Stones</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Wealth</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>F vs F</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>2d8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>2d6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Force 6</t>
+          <t>Wealth 3, Magic 2</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Special</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Sunken Heart</t>
+          <t>Veins frontier</t>
         </is>
       </c>
     </row>
@@ -5333,38 +5333,38 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Heavy Infantry</t>
+          <t>Bound Spirit</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Force</t>
+          <t>Magic</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>F vs F</t>
+          <t>M vs F</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>1d10</t>
+          <t>1d8</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>1d8</t>
+          <t>1d6</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Force 3</t>
+          <t>Magic 3</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -5940,7 +5940,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Merchant Princes</t>
+          <t>Maze-Toll</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -5949,39 +5949,39 @@
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>W vs W</t>
+          <t>W vs M</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>2d6</t>
+          <t>1d6</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>1d8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Wealth 6</t>
+          <t>Wealth 4, Magic 3</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Special</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Trade-Vein hubs</t>
+          <t>Each maze entrance</t>
         </is>
       </c>
     </row>
@@ -6036,96 +6036,96 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Bound Spirit</t>
+          <t>Janeen Aesthete-Spies</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Magic</t>
+          <t>Cunning</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
         <v>8</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>M vs F</t>
+          <t>C vs C</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>1d8</t>
+          <t>1d10</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>1d6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Magic 3</t>
+          <t>Cunning 4, Magic 2</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Subtle</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Each maze entrance</t>
+          <t>Surface and underdark salons</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Seductive Cabal</t>
+          <t>Bound Spirit</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Cunning</t>
+          <t>Magic</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>C vs C</t>
+          <t>M vs F</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>1d10</t>
+          <t>1d8</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>Magic 3</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>Cunning 5</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>Subtle</t>
-        </is>
-      </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Surface and underdark salons</t>
+          <t>Janeen frontier</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6691,7 +6691,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Brigand Cell</t>
+          <t>Olm Listeners</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -6703,11 +6703,11 @@
         <v>2</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>C vs F</t>
+          <t>C vs C</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -6717,7 +6717,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>1d4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -6727,277 +6727,325 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Stealthed</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Wherever a recent battle left bodies</t>
+          <t>Drowned Galleries</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Hedge Mages</t>
+          <t>Hidden Larder</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Magic</t>
+          <t>Wealth</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D30" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>M vs M</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>1d6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>1d4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Magic 1</t>
+          <t>Wealth 1</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Stealthed, Special</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Drowned Galleries</t>
+          <t>Concealed gallery niches</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
+          <t>Olm Anatomist</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>M vs F</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>2d4</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Magic 3</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Stealthed, Special</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>Drowned Galleries</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
           <t>Spirit Walkers</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Magic</t>
         </is>
       </c>
-      <c r="C31" s="5" t="n">
+      <c r="C32" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D31" s="5" t="n">
+      <c r="D32" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>M vs C</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>1d6</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>Magic 2</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr">
         <is>
           <t>Stealthed, Subtle</t>
         </is>
       </c>
-      <c r="J31" s="5" t="inlineStr">
+      <c r="J32" s="6" t="inlineStr">
         <is>
           <t>Deep pools</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="19" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="34" ht="19" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Turn Log (fill as you play)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Turn</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>Treasure +/–</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Action Taken</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>Goal Progress</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="5" t="n">
+    <row r="36">
+      <c r="A36" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B35" s="5" t="inlineStr"/>
-      <c r="C35" s="5" t="inlineStr"/>
-      <c r="D35" s="5" t="inlineStr"/>
-      <c r="E35" s="5" t="inlineStr"/>
-      <c r="F35" s="5" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="n">
+      <c r="B36" s="5" t="inlineStr"/>
+      <c r="C36" s="5" t="inlineStr"/>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B36" s="6" t="inlineStr"/>
-      <c r="C36" s="6" t="inlineStr"/>
-      <c r="D36" s="6" t="inlineStr"/>
-      <c r="E36" s="6" t="inlineStr"/>
-      <c r="F36" s="6" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="n">
+      <c r="B37" s="6" t="inlineStr"/>
+      <c r="C37" s="6" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B37" s="5" t="inlineStr"/>
-      <c r="C37" s="5" t="inlineStr"/>
-      <c r="D37" s="5" t="inlineStr"/>
-      <c r="E37" s="5" t="inlineStr"/>
-      <c r="F37" s="5" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="n">
+      <c r="B38" s="5" t="inlineStr"/>
+      <c r="C38" s="5" t="inlineStr"/>
+      <c r="D38" s="5" t="inlineStr"/>
+      <c r="E38" s="5" t="inlineStr"/>
+      <c r="F38" s="5" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B38" s="6" t="inlineStr"/>
-      <c r="C38" s="6" t="inlineStr"/>
-      <c r="D38" s="6" t="inlineStr"/>
-      <c r="E38" s="6" t="inlineStr"/>
-      <c r="F38" s="6" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="n">
+      <c r="B39" s="6" t="inlineStr"/>
+      <c r="C39" s="6" t="inlineStr"/>
+      <c r="D39" s="6" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr"/>
+      <c r="F39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B39" s="5" t="inlineStr"/>
-      <c r="C39" s="5" t="inlineStr"/>
-      <c r="D39" s="5" t="inlineStr"/>
-      <c r="E39" s="5" t="inlineStr"/>
-      <c r="F39" s="5" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="n">
+      <c r="B40" s="5" t="inlineStr"/>
+      <c r="C40" s="5" t="inlineStr"/>
+      <c r="D40" s="5" t="inlineStr"/>
+      <c r="E40" s="5" t="inlineStr"/>
+      <c r="F40" s="5" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B40" s="6" t="inlineStr"/>
-      <c r="C40" s="6" t="inlineStr"/>
-      <c r="D40" s="6" t="inlineStr"/>
-      <c r="E40" s="6" t="inlineStr"/>
-      <c r="F40" s="6" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="n">
+      <c r="B41" s="6" t="inlineStr"/>
+      <c r="C41" s="6" t="inlineStr"/>
+      <c r="D41" s="6" t="inlineStr"/>
+      <c r="E41" s="6" t="inlineStr"/>
+      <c r="F41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B41" s="5" t="inlineStr"/>
-      <c r="C41" s="5" t="inlineStr"/>
-      <c r="D41" s="5" t="inlineStr"/>
-      <c r="E41" s="5" t="inlineStr"/>
-      <c r="F41" s="5" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="n">
+      <c r="B42" s="5" t="inlineStr"/>
+      <c r="C42" s="5" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr"/>
+      <c r="F42" s="5" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B42" s="6" t="inlineStr"/>
-      <c r="C42" s="6" t="inlineStr"/>
-      <c r="D42" s="6" t="inlineStr"/>
-      <c r="E42" s="6" t="inlineStr"/>
-      <c r="F42" s="6" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="n">
+      <c r="B43" s="6" t="inlineStr"/>
+      <c r="C43" s="6" t="inlineStr"/>
+      <c r="D43" s="6" t="inlineStr"/>
+      <c r="E43" s="6" t="inlineStr"/>
+      <c r="F43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B43" s="5" t="inlineStr"/>
-      <c r="C43" s="5" t="inlineStr"/>
-      <c r="D43" s="5" t="inlineStr"/>
-      <c r="E43" s="5" t="inlineStr"/>
-      <c r="F43" s="5" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="n">
+      <c r="B44" s="5" t="inlineStr"/>
+      <c r="C44" s="5" t="inlineStr"/>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B44" s="6" t="inlineStr"/>
-      <c r="C44" s="6" t="inlineStr"/>
-      <c r="D44" s="6" t="inlineStr"/>
-      <c r="E44" s="6" t="inlineStr"/>
-      <c r="F44" s="6" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="n">
+      <c r="B45" s="6" t="inlineStr"/>
+      <c r="C45" s="6" t="inlineStr"/>
+      <c r="D45" s="6" t="inlineStr"/>
+      <c r="E45" s="6" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B45" s="5" t="inlineStr"/>
-      <c r="C45" s="5" t="inlineStr"/>
-      <c r="D45" s="5" t="inlineStr"/>
-      <c r="E45" s="5" t="inlineStr"/>
-      <c r="F45" s="5" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="n">
+      <c r="B46" s="5" t="inlineStr"/>
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr"/>
+      <c r="F46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B46" s="6" t="inlineStr"/>
-      <c r="C46" s="6" t="inlineStr"/>
-      <c r="D46" s="6" t="inlineStr"/>
-      <c r="E46" s="6" t="inlineStr"/>
-      <c r="F46" s="6" t="inlineStr"/>
+      <c r="B47" s="6" t="inlineStr"/>
+      <c r="C47" s="6" t="inlineStr"/>
+      <c r="D47" s="6" t="inlineStr"/>
+      <c r="E47" s="6" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A33:F33"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A34:F34"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A25:F25"/>
   </mergeCells>
@@ -7981,17 +8029,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
@@ -10783,13 +10831,1405 @@
         </is>
       </c>
     </row>
+    <row r="68" ht="19" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Setting Assets — Veins of the Earth (Force)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="28" customHeight="1">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>Attack (Atk vs Def)</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Damage</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>Counter</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>Min Attr</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>Traits</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>Notes / Special</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>Tunnel Crawlers</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D70" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>F vs F</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>1d4</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>Force 2</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>Light infantry trained for narrow ways; Move cost ignored within the Veins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>Lantern Wardens</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>F vs M</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>1d8</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t>1d4</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>Force 3</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J71" s="6" t="inlineStr">
+        <is>
+          <t>Gnonmen heavy-light bearers. While present, rival Magic and Stealthed attacks in this location are at -1 to the roll.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Stone-Eaters</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D72" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>F vs F</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>1d10</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>1d8</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>Force 4, Magic 2</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>Substratal close-order elementals. Halve all damage from non-Magic attacks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>Crystal Lancers</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D73" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>F vs M</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>1d10</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>Force 3, Magic 1</t>
+        </is>
+      </c>
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J73" s="6" t="inlineStr">
+        <is>
+          <t>dErO troops with crackling polearms. Double damage vs Magic assets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>Spore-Maddened Slaves</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D74" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>F vs F</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>Force 2</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>Fanatic</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>Funginid spore-controlled bodies. Cannot retreat and cannot be Healed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>Dream-Knights of the Black Glass Court</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>F vs C</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>2d6</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>1d10</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>Force 5, Magic 2</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J75" s="6" t="inlineStr">
+        <is>
+          <t>Aelf-Adal household champions. +1 to attack rolls vs locations under any Cult Network.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="19" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Setting Assets — Veins of the Earth (Cunning)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="28" customHeight="1">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Attack (Atk vs Def)</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Damage</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>Counter</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>Min Attr</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>Traits</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>Notes / Special</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>Spore-Wreaths</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Cunning</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D79" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>C vs C</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>Cunning 2</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>Stealthed, Subtle</t>
+        </is>
+      </c>
+      <c r="J79" s="5" t="inlineStr">
+        <is>
+          <t>Funginid spy-mats. If destroyed in a location with another Funginid asset, re-roots at 1 HP next turn at no cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>Lightless Cartographers</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>Cunning</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D80" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>C vs C</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>1d4</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>Cunning 1</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>Stealthed, Mobile</t>
+        </is>
+      </c>
+      <c r="J80" s="6" t="inlineStr">
+        <is>
+          <t>Veins mapmakers. Once per turn, reveal one unexplored adjacent location to the owning faction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>Debt-Collectors</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Cunning</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D81" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>C vs W</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>1d8</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>Cunning 2, Magic 1</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>Subtle</t>
+        </is>
+      </c>
+      <c r="J81" s="5" t="inlineStr">
+        <is>
+          <t>Knotsmen with infernally binding scrolls. On a successful attack, owner gains 1 Treasure instead of (or in addition to) inflicting the last 2 damage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>Dream-Walkers</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>Cunning</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D82" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>C vs M</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>1d8</t>
+        </is>
+      </c>
+      <c r="G82" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>Cunning 3, Magic 2</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>Stealthed, Subtle</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="inlineStr">
+        <is>
+          <t>Aelf-Adal subconscious infiltrators. May attack any asset in a location that contains a Cult Network, regardless of distance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>Olm Listeners</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Cunning</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D83" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>C vs C</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>Cunning 1</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>Stealthed</t>
+        </is>
+      </c>
+      <c r="J83" s="5" t="inlineStr">
+        <is>
+          <t>Silent amphibians pressed to wet stone. Free action: on 4+ on 1d6, learn one rival action declared this turn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>Janeen Aesthete-Spies</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Cunning</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D84" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E84" s="6" t="inlineStr">
+        <is>
+          <t>C vs C</t>
+        </is>
+      </c>
+      <c r="F84" s="6" t="inlineStr">
+        <is>
+          <t>1d10</t>
+        </is>
+      </c>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>Cunning 4, Magic 2</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>Subtle</t>
+        </is>
+      </c>
+      <c r="J84" s="6" t="inlineStr">
+        <is>
+          <t>Deep Janeen connoisseur-intelligencers. Each turn, reveal one tag of a rival faction (may also be used as polite blackmail).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="19" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Setting Assets — Veins of the Earth (Wealth)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="28" customHeight="1">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>Attack (Atk vs Def)</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>Damage</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>Counter</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>Min Attr</t>
+        </is>
+      </c>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>Traits</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>Notes / Special</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>Mushroom Fields</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Wealth</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D88" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>W vs W</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>1d4</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>1d4</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>Wealth 2</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>Gnonmen subsistence cultivation. On 4+ on 1d6 at turn start, gain 1 Treasure. Any fire or scour attack deals +3 damage to this asset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>Pact-Vaults</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>Wealth</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D89" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E89" s="6" t="inlineStr">
+        <is>
+          <t>W vs W</t>
+        </is>
+      </c>
+      <c r="F89" s="6" t="inlineStr">
+        <is>
+          <t>1d8</t>
+        </is>
+      </c>
+      <c r="G89" s="6" t="inlineStr">
+        <is>
+          <t>1d4</t>
+        </is>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>Wealth 4, Magic 1</t>
+        </is>
+      </c>
+      <c r="I89" s="6" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J89" s="6" t="inlineStr">
+        <is>
+          <t>Knotsmen infernal banking. Stockpiles up to 6 Treasure. If destroyed, the stored Treasure is lost AND the attacker's nearest Wealth asset takes 2d6 damage from vengeful contract-fiends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>Crystal Mines</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Wealth</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D90" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>W vs F</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>Wealth 3, Magic 1</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr">
+        <is>
+          <t>dErO industrial workings. +1 Treasure per turn; reduces the Cost of Magic assets built at this location by 1 (min 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>Maze-Toll</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>Wealth</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D91" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>W vs M</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="inlineStr">
+        <is>
+          <t>Wealth 4, Magic 3</t>
+        </is>
+      </c>
+      <c r="I91" s="6" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J91" s="6" t="inlineStr">
+        <is>
+          <t>Deep Janeen labyrinth-entry. +2 Treasure per turn while undisturbed; collapses (asset destroyed) if any rival Magic asset enters the location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>Hidden Larder</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Wealth</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D92" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>Wealth 1</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>Stealthed, Special</t>
+        </is>
+      </c>
+      <c r="J92" s="5" t="inlineStr">
+        <is>
+          <t>Olm food caches squirreled into wet stone. Spend 1 Treasure as a free action to bring one of your destroyed non-Magic 1-cost assets back at 1 HP in this location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>Substratal Tribute Stones</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>Wealth</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D93" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E93" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G93" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>Wealth 3, Magic 2</t>
+        </is>
+      </c>
+      <c r="I93" s="6" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J93" s="6" t="inlineStr">
+        <is>
+          <t>Geomantic tax-pillars. Generates +1 Treasure per turn for every Magic asset that shares this location, including rivals'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="19" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Setting Assets — Veins of the Earth (Magic)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="28" customHeight="1">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>Attack (Atk vs Def)</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>Damage</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>Counter</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>Min Attr</t>
+        </is>
+      </c>
+      <c r="I96" s="4" t="inlineStr">
+        <is>
+          <t>Traits</t>
+        </is>
+      </c>
+      <c r="J96" s="4" t="inlineStr">
+        <is>
+          <t>Notes / Special</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>Spore-Cathedral Choir</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D97" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>M vs M</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>1d8</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>Magic 3</t>
+        </is>
+      </c>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J97" s="5" t="inlineStr">
+        <is>
+          <t>Funginid ritualists. At start of each turn, heal 1 HP to every Funginid Cunning asset in this location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>Dream Anchor</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D98" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>M vs M</t>
+        </is>
+      </c>
+      <c r="F98" s="6" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="G98" s="6" t="inlineStr">
+        <is>
+          <t>1d8</t>
+        </is>
+      </c>
+      <c r="H98" s="6" t="inlineStr">
+        <is>
+          <t>Magic 4</t>
+        </is>
+      </c>
+      <c r="I98" s="6" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J98" s="6" t="inlineStr">
+        <is>
+          <t>Aelf-Adal sleeping-relic. Rival Magic actions in this location cost +1 Treasure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>Demonic Notary</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D99" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>M vs M</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>1d10</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="H99" s="5" t="inlineStr">
+        <is>
+          <t>Magic 3</t>
+        </is>
+      </c>
+      <c r="I99" s="5" t="inlineStr">
+        <is>
+          <t>Subtle, Special</t>
+        </is>
+      </c>
+      <c r="J99" s="5" t="inlineStr">
+        <is>
+          <t>Knotsmen pact-fiend. Once per turn, force any rival to pay 1 Treasure or cancel an action declared against your faction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>Hearth-Lantern Shrine</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D100" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E100" s="6" t="inlineStr">
+        <is>
+          <t>M vs M</t>
+        </is>
+      </c>
+      <c r="F100" s="6" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="G100" s="6" t="inlineStr">
+        <is>
+          <t>1d4</t>
+        </is>
+      </c>
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t>Magic 2</t>
+        </is>
+      </c>
+      <c r="I100" s="6" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J100" s="6" t="inlineStr">
+        <is>
+          <t>Gnonmen warding-light. Stealthed assets in this location are revealed automatically; the light does not permit hiding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>Stone-Voice Oracle</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D101" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>M vs M</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>1d8</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>1d8</t>
+        </is>
+      </c>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t>Magic 4</t>
+        </is>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="J101" s="5" t="inlineStr">
+        <is>
+          <t>Substratal seer-elemental. At start of each turn, the owner may force one rival to declare their action before declaring their own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>Olm Anatomist</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D102" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E102" s="6" t="inlineStr">
+        <is>
+          <t>M vs F</t>
+        </is>
+      </c>
+      <c r="F102" s="6" t="inlineStr">
+        <is>
+          <t>2d4</t>
+        </is>
+      </c>
+      <c r="G102" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t>Magic 3</t>
+        </is>
+      </c>
+      <c r="I102" s="6" t="inlineStr">
+        <is>
+          <t>Stealthed, Special</t>
+        </is>
+      </c>
+      <c r="J102" s="6" t="inlineStr">
+        <is>
+          <t>Knower of unmaking-shapes. Deals double damage to any asset with HP 6 or less.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="9">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A37:J37"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A21:J21"/>
+    <mergeCell ref="A77:J77"/>
+    <mergeCell ref="A95:J95"/>
     <mergeCell ref="A54:J54"/>
+    <mergeCell ref="A86:J86"/>
+    <mergeCell ref="A68:J68"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12578,7 +14018,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Counting House</t>
+          <t>Pact-Vaults</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -12587,10 +14027,10 @@
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
@@ -12599,22 +14039,22 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>1d10</t>
+          <t>1d8</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>1d6</t>
+          <t>1d4</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Wealth 5</t>
+          <t>Wealth 4, Magic 1</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Special</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
@@ -12626,7 +14066,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Spies</t>
+          <t>Debt-Collectors</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -12635,19 +14075,19 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>C vs C</t>
+          <t>C vs W</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>1d6</t>
+          <t>1d8</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -12657,12 +14097,12 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Cunning 2</t>
+          <t>Cunning 2, Magic 1</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>Stealthed, Subtle</t>
+          <t>Subtle</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
@@ -12674,7 +14114,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Demonologists</t>
+          <t>Demonic Notary</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -12683,11 +14123,11 @@
         </is>
       </c>
       <c r="C31" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D31" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="D31" s="5" t="n">
-        <v>8</v>
-      </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
           <t>M vs M</t>
@@ -12700,7 +14140,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>1d4</t>
+          <t>1d6</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -12710,7 +14150,7 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Subtle</t>
+          <t>Subtle, Special</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Canonicalise faction locations to the campaign's named places
Updates each of the nine factions' HQ and asset locations to use the
canonical Veins-of-the-Earth places: Celephais (Aelf-Adal), Gordiam
(Knotsmen), Comorragh (Dvargir), Piranesi (Deep Janeen), Genet
(Funginids), The Core (Substratals), Heliotropolis (Gnonmen), Nox
(shared trade city), Isles of the Imprisoned Moon (contested - dErO and
Olm both press here). dErO and Olm have no fixed capital; their assets
are spread across Nox and the Isles.

Adds a LOCATIONS constant and the DefinedName import in preparation for
the upcoming automation sheets (Asset Register, Locations Matrix,
Action Sheet, Turn Summary) that will use these as their location set.
</commit_message>
<xml_diff>
--- a/WWN_Veins_of_the_Earth_Factions.xlsx
+++ b/WWN_Veins_of_the_Earth_Factions.xlsx
@@ -1013,7 +1013,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>The Hall of Mirroring Dreams</t>
+          <t>Celephais</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Multiple surface courts</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Mirror Halls</t>
+          <t>Celephais</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Veins waystations</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Mirror Halls</t>
+          <t>Celephais</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Mirror Halls</t>
+          <t>Celephais</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Black Glass Court</t>
+          <t>Celephais</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Sleeping Sanctum</t>
+          <t>Celephais</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>The Spore-Cathedral</t>
+          <t>Genet</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Slave-pens across the Veins</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Every slave market</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Cattle-races' larders</t>
+          <t>Genet</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Spore-Cathedral</t>
+          <t>Genet</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Carrion grounds</t>
+          <t>Genet</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Spore-Cathedral</t>
+          <t>Genet</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2563,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>The Buzzing Halls</t>
+          <t>No fixed capital — cells across the Veins</t>
         </is>
       </c>
     </row>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Buzzing Halls</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Crystal Pylons</t>
+          <t>Isles of the Imprisoned Moon</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Crystal Pylons</t>
+          <t>Isles of the Imprisoned Moon</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Surface intelligence services</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Lower Buzzing Halls</t>
+          <t>Isles of the Imprisoned Moon</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Buzzing Halls</t>
+          <t>Isles of the Imprisoned Moon</t>
         </is>
       </c>
     </row>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Across the Veins</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Forgeholds of Anvil-Below</t>
+          <t>Comorragh</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Forgeholds</t>
+          <t>Comorragh</t>
         </is>
       </c>
     </row>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Forgeholds</t>
+          <t>Comorragh</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Forgeholds</t>
+          <t>Comorragh</t>
         </is>
       </c>
     </row>
@@ -3680,7 +3680,7 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Caravan routes</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Forgeholds</t>
+          <t>Comorragh</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Anvil-Below</t>
+          <t>Comorragh</t>
         </is>
       </c>
     </row>
@@ -3824,7 +3824,7 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Vassal warrens</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>The Lantern Holds</t>
+          <t>Heliotropolis</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Lantern Holds</t>
+          <t>Heliotropolis</t>
         </is>
       </c>
     </row>
@@ -4383,7 +4383,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Veins patrol routes</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Lantern Holds</t>
+          <t>Heliotropolis</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Surface of the Lantern Holds</t>
+          <t>Heliotropolis</t>
         </is>
       </c>
     </row>
@@ -4527,7 +4527,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Lantern Holds</t>
+          <t>Heliotropolis</t>
         </is>
       </c>
     </row>
@@ -4575,7 +4575,7 @@
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Across Gnonmen friend-networks</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Upper passes</t>
+          <t>Heliotropolis</t>
         </is>
       </c>
     </row>
@@ -4960,7 +4960,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>The Sunken Heart</t>
+          <t>The Core</t>
         </is>
       </c>
     </row>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Sunken Heart</t>
+          <t>The Core</t>
         </is>
       </c>
     </row>
@@ -5182,7 +5182,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Sunken Heart</t>
+          <t>The Core</t>
         </is>
       </c>
     </row>
@@ -5230,7 +5230,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Veins frontier</t>
+          <t>The Core</t>
         </is>
       </c>
     </row>
@@ -5278,7 +5278,7 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Stone-fields</t>
+          <t>The Core</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Sunken Heart</t>
+          <t>The Core</t>
         </is>
       </c>
     </row>
@@ -5374,7 +5374,7 @@
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Substratal frontier</t>
+          <t>Comorragh</t>
         </is>
       </c>
     </row>
@@ -5711,7 +5711,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Each in their own maze</t>
+          <t>Piranesi</t>
         </is>
       </c>
     </row>
@@ -5885,7 +5885,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Their personal maze</t>
+          <t>Piranesi</t>
         </is>
       </c>
     </row>
@@ -5933,7 +5933,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Janeen courts</t>
+          <t>Piranesi</t>
         </is>
       </c>
     </row>
@@ -5981,7 +5981,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Each maze entrance</t>
+          <t>Piranesi</t>
         </is>
       </c>
     </row>
@@ -6029,7 +6029,7 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Janeen courts</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -6077,7 +6077,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Surface and underdark salons</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -6125,7 +6125,7 @@
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Janeen frontier</t>
+          <t>Piranesi</t>
         </is>
       </c>
     </row>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>The Drowned Galleries</t>
+          <t>No fixed capital — wanders the drowned routes</t>
         </is>
       </c>
     </row>
@@ -6636,7 +6636,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Drowned Galleries</t>
+          <t>Isles of the Imprisoned Moon</t>
         </is>
       </c>
     </row>
@@ -6684,7 +6684,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Underwater Vein routes</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -6732,7 +6732,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Drowned Galleries</t>
+          <t>Isles of the Imprisoned Moon</t>
         </is>
       </c>
     </row>
@@ -6780,7 +6780,7 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Concealed gallery niches</t>
+          <t>Isles of the Imprisoned Moon</t>
         </is>
       </c>
     </row>
@@ -6828,7 +6828,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Drowned Galleries</t>
+          <t>Isles of the Imprisoned Moon</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Deep pools</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -13789,7 +13789,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>The Compounding Vaults</t>
+          <t>Gordiam</t>
         </is>
       </c>
     </row>
@@ -13963,7 +13963,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Mid-Veins markets</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -14011,7 +14011,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Compounding Vaults</t>
+          <t>Gordiam</t>
         </is>
       </c>
     </row>
@@ -14059,7 +14059,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Compounding Vaults</t>
+          <t>Gordiam</t>
         </is>
       </c>
     </row>
@@ -14107,7 +14107,7 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Surface debtor towns</t>
+          <t>Nox</t>
         </is>
       </c>
     </row>
@@ -14155,7 +14155,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Hall of Contracts</t>
+          <t>Gordiam</t>
         </is>
       </c>
     </row>
@@ -14203,7 +14203,7 @@
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Compounding Vaults</t>
+          <t>Gordiam</t>
         </is>
       </c>
     </row>
@@ -14251,7 +14251,7 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Rival faction debt-houses</t>
+          <t>Comorragh</t>
         </is>
       </c>
     </row>

</xml_diff>